<commit_message>
auto: snapshot from claude session
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2571,6 +2571,1308 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Follow up with Aman about payment issue</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Reach out to Aman to clarify the payment issue and confirm the details of the purchase.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>To resolve the payment issue and ensure customer satisfaction.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Anchit</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Configure Growth Pillar</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Configure the growth pillar with the correct name, SPOC, and priority. Ensure it is correctly categorized under Growth, Color, Retention, Acquisition.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>To accurately track and measure growth metrics.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Update the sheet with old content</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Add the old content to the new sheet, and make sure it's not mixed with new content.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>To ensure that the new sheet is accurate and easy to use.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Update status in OOSI</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Add a new status to OOSI to track progress and avoid mixing tasks.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>To improve task management and avoid confusion.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Implement WhatsApp APIs</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Explore and implement WhatsApp APIs to integrate with Vahdam India's systems.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>To leverage WhatsApp for customer engagement and communication.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Retention</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Explore Google Chat API</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Anchit wants to use Google Chat API for automation, as it's free and can be used in place of WhatsApp Business API.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Using Google Chat API can simplify automation and reduce costs.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Anchit</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Create Automated Tracker Project</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Develop an automated tracker project to improve efficiency and accuracy.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>To streamline processes and reduce manual errors.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Create Automated Tracker Project</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Develop an automated tracker project to improve efficiency and accuracy.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>To streamline processes and reduce manual errors.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Verify Landing Page Status</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Check the status of the landing pages, including the final URLs, and ensure they are ready to go live by the 6th of May.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>6th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Review Dashboard Status</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Verify the production use of the dashboard and ensure it is ready by the 7th of May.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>7th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Finalize Creator Partnerships</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Finalize the cadence of creator partnerships and ensure it is completed by the 7th of May.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>7th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Review Pagedeck Status</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Verify the Pagedeck live on the website and ensure it is ready by the 6th of May.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>6th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Review Dashboard Progress</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Verify the progress of the production use of the dashboard and ensure it is completed by the specified timeline.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>To ensure timely completion of the dashboard and avoid delays in marketing efforts.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>7th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Schedule Landing Page Experts Conversation</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Schedule a final conversation with landing page experts and ensure it is completed by the specified timeline.</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>To gather expert insights and drive marketing efforts.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Brand &amp; Content</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>13th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Review and address feedback from second meeting with Akhil</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Review the feedback from the second meeting with Akhil and address any errors or issues mentioned.</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>To ensure that the feedback is addressed and to improve the overall quality of the meeting.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Anchit</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Check lending page buttons</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Verify that the lending page buttons are working properly and troubleshoot any issues. Provide a detailed report to Aman Gupta.</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>The lending page buttons not working is a critical issue that needs to be resolved to ensure a smooth user experience.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Review and confirm updated timelines</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Review the updated timelines provided by Aman Gupta and confirm that all tasks are on track to meet the deadlines.</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>The updated timelines are crucial to ensure that all tasks are completed on time and that the project stays on track.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Follow up with Aman on lending page issues</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Reach out to Aman Gupta to confirm the status of the lending page buttons and ensure that the issue is resolved.</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>To maintain open communication and ensure that the issue is addressed promptly.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Anchit Tandon</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Check lending page buttons</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Verify that the lending page buttons are working properly and troubleshoot any issues. Provide a detailed report to Aman Gupta.</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>The lending page buttons not working is a critical issue that needs to be resolved to ensure a smooth user experience.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Review and confirm updated timelines</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Review the updated timelines provided by Aman Gupta and confirm that all tasks are on track to meet the deadlines.</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>The updated timelines are crucial to ensure that all tasks are completed on time and that the project stays on track.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Follow up with Aman on lending page issues</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Reach out to Aman Gupta to confirm the status of the lending page buttons and ensure that the issue is resolved.</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>To maintain open communication and ensure that the issue is addressed promptly.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Anchit Tandon</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Check and fix PDP page code</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Aman needs to investigate and resolve the issue with the PDP page not loading, despite HTML working fine. He should check the code and provide a solution to Anchit.</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>The PDP page issue is blocking sales and customer experience. Aman needs to resolve this ASAP to prevent further delays.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Troubleshoot PDP issues on Shopify</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Work with Aman to identify and fix the issues with the PDP on Shopify, specifically with HTML, CODI, and Copy.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Fixing the PDP issues will improve the customer experience and potentially increase conversion rates.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Conversion</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Check and fix PDP page code</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Aman needs to investigate and resolve the issue with the PDP page not loading, despite HTML working fine. He should check the code and provide a solution to Anchit.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>The PDP page issue is blocking sales and customer experience. Aman needs to resolve this ASAP to prevent further delays.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Troubleshoot PDP issues on Shopify</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Work with Aman to identify and fix the issues with the PDP on Shopify, specifically with HTML, CODI, and Copy.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Fixing the PDP issues will improve the customer experience and potentially increase conversion rates.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Conversion</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Add email data to MOM report</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Include email data, cancellations flows, and winback data in the MOM report as requested by Akhil Arora.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>To provide a comprehensive view of the business performance.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Retention</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Check lending page buttons</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Verify that the lending page buttons are working properly and fix any issues found.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>To ensure a smooth user experience on the lending page.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Implement Note-Taking and Task-Making System</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Create a system to store notes and tasks from various sources (discussions, meetings, Gmail, WhatsApp) in a centralized location (Google Sheets, Excel, WhatsApp chat) with status update options.</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Chat | DM</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>To improve organization and productivity by having a single source of truth for notes and tasks.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Team &amp; Process</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Implement Note-Taking and Task-Making System</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Create a system to store notes and tasks from various sources (discussions, meetings, emails, chats, spaces, groups, WhatsApp chats) in a centralized location (Google Sheets and Excel file) with status update options.</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Chat | DM</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>To improve productivity and organization by having a single source of truth for notes and tasks.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Team &amp; Process</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Fix HTML coding issue on page deck</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Check and resolve the issue where something doesn't display on the page deck due to HTML coding in the HTML file.</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Fixing this issue will improve the user experience and ensure that all content is displayed correctly on the page deck.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2582,7 +3884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -4768,6 +6070,688 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Follow up with Aman about payment issue</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Reach out to Aman to clarify the payment issue and confirm the details of the purchase.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>To resolve the payment issue and ensure customer satisfaction.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Anchit</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Configure Growth Pillar</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Configure the growth pillar with the correct name, SPOC, and priority. Ensure it is correctly categorized under Growth, Color, Retention, Acquisition.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>To accurately track and measure growth metrics.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Update the sheet with old content</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Add the old content to the new sheet, and make sure it's not mixed with new content.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>To ensure that the new sheet is accurate and easy to use.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Update status in OOSI</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Add a new status to OOSI to track progress and avoid mixing tasks.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>To improve task management and avoid confusion.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Implement WhatsApp APIs</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Explore and implement WhatsApp APIs to integrate with Vahdam India's systems.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>To leverage WhatsApp for customer engagement and communication.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Retention</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Explore Google Chat API</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Anchit wants to use Google Chat API for automation, as it's free and can be used in place of WhatsApp Business API.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Using Google Chat API can simplify automation and reduce costs.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Anchit</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Create Automated Tracker Project</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Develop an automated tracker project to improve efficiency and accuracy.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>To streamline processes and reduce manual errors.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Create Automated Tracker Project</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Develop an automated tracker project to improve efficiency and accuracy.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>To streamline processes and reduce manual errors.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Review and address feedback from second meeting with Akhil</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Review the feedback from the second meeting with Akhil and address any errors or issues mentioned.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>To ensure that the feedback is addressed and to improve the overall quality of the meeting.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Anchit</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Check and fix PDP page code</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Aman needs to investigate and resolve the issue with the PDP page not loading, despite HTML working fine. He should check the code and provide a solution to Anchit.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>The PDP page issue is blocking sales and customer experience. Aman needs to resolve this ASAP to prevent further delays.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Troubleshoot PDP issues on Shopify</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Work with Aman to identify and fix the issues with the PDP on Shopify, specifically with HTML, CODI, and Copy.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Fixing the PDP issues will improve the customer experience and potentially increase conversion rates.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Conversion</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Check and fix PDP page code</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Aman needs to investigate and resolve the issue with the PDP page not loading, despite HTML working fine. He should check the code and provide a solution to Anchit.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>The PDP page issue is blocking sales and customer experience. Aman needs to resolve this ASAP to prevent further delays.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Troubleshoot PDP issues on Shopify</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Work with Aman to identify and fix the issues with the PDP on Shopify, specifically with HTML, CODI, and Copy.</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Fixing the PDP issues will improve the customer experience and potentially increase conversion rates.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Conversion</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Implement Note-Taking and Task-Making System</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Create a system to store notes and tasks from various sources (discussions, meetings, Gmail, WhatsApp) in a centralized location (Google Sheets, Excel, WhatsApp chat) with status update options.</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Chat | DM</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>To improve organization and productivity by having a single source of truth for notes and tasks.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Team &amp; Process</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Implement Note-Taking and Task-Making System</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Create a system to store notes and tasks from various sources (discussions, meetings, emails, chats, spaces, groups, WhatsApp chats) in a centralized location (Google Sheets and Excel file) with status update options.</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Chat | DM</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>To improve productivity and organization by having a single source of truth for notes and tasks.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Team &amp; Process</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Fix HTML coding issue on page deck</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Check and resolve the issue where something doesn't display on the page deck due to HTML coding in the HTML file.</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Meeting | voice memo by Anchit (Self)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Fixing this issue will improve the user experience and ensure that all content is displayed correctly on the page deck.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4779,7 +6763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -4846,6 +6830,624 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Verify Landing Page Status</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Check the status of the landing pages, including the final URLs, and ensure they are ready to go live by the 6th of May.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>6th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Review Dashboard Status</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Verify the production use of the dashboard and ensure it is ready by the 7th of May.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>7th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Finalize Creator Partnerships</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Finalize the cadence of creator partnerships and ensure it is completed by the 7th of May.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>7th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Review Pagedeck Status</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Verify the Pagedeck live on the website and ensure it is ready by the 6th of May.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>To ensure timely launch and meet the marketing goals.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>6th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Review Dashboard Progress</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Verify the progress of the production use of the dashboard and ensure it is completed by the specified timeline.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>To ensure timely completion of the dashboard and avoid delays in marketing efforts.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>7th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Schedule Landing Page Experts Conversation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Schedule a final conversation with landing page experts and ensure it is completed by the specified timeline.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>To gather expert insights and drive marketing efforts.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Brand &amp; Content</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>13th May</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Check lending page buttons</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Verify that the lending page buttons are working properly and troubleshoot any issues. Provide a detailed report to Aman Gupta.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>The lending page buttons not working is a critical issue that needs to be resolved to ensure a smooth user experience.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Review and confirm updated timelines</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Review the updated timelines provided by Aman Gupta and confirm that all tasks are on track to meet the deadlines.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>The updated timelines are crucial to ensure that all tasks are completed on time and that the project stays on track.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Follow up with Aman on lending page issues</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Reach out to Aman Gupta to confirm the status of the lending page buttons and ensure that the issue is resolved.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>To maintain open communication and ensure that the issue is addressed promptly.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Anchit Tandon</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Check lending page buttons</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Verify that the lending page buttons are working properly and troubleshoot any issues. Provide a detailed report to Aman Gupta.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>The lending page buttons not working is a critical issue that needs to be resolved to ensure a smooth user experience.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Review and confirm updated timelines</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Review the updated timelines provided by Aman Gupta and confirm that all tasks are on track to meet the deadlines.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>The updated timelines are crucial to ensure that all tasks are completed on time and that the project stays on track.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Akhil Arora</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Follow up with Aman on lending page issues</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Reach out to Aman Gupta to confirm the status of the lending page buttons and ensure that the issue is resolved.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>To maintain open communication and ensure that the issue is addressed promptly.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Anchit Tandon</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Add email data to MOM report</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Include email data, cancellations flows, and winback data in the MOM report as requested by Akhil Arora.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>To provide a comprehensive view of the business performance.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Retention</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Check lending page buttons</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Verify that the lending page buttons are working properly and fix any issues found.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Email | from Akhil Arora</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>To ensure a smooth user experience on the lending page.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Aman Gupta</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>